<commit_message>
feat(pib): ajustes finales de ficha PIB oportuno para merge
- Filtros históricos por número exacto de observaciones trimestrales (1a=4, 2a=8, 3a=12, 5a=20).
- Historial compacto: periodo inicial, periodo final y total de observaciones.
- Lectura del indicador con 4 bullets dinámicos y sin próxima publicación.
- Excel PIB separado en hojas "PIB oportuno" y "Nivel PIB".
- Tests validan cobertura EOPIBT, separación PIBT, actividades y formato Excel.

Generated with [Devin](https://devin.ai)
</commit_message>
<xml_diff>
--- a/downloads/indicadores/IOAE/IOAE_datos.xlsx
+++ b/downloads/indicadores/IOAE/IOAE_datos.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>URL del boletín / serie: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf · Fecha de publicación: 21 de julio de 2026</t>
+          <t>URL del boletín / serie: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf · Fecha de publicación: 20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -623,12 +623,12 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -681,12 +681,12 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -739,12 +739,12 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -797,12 +797,12 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1029,12 +1029,12 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1087,12 +1087,12 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1145,12 +1145,12 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1203,12 +1203,12 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1261,12 +1261,12 @@
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1377,12 +1377,12 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1435,12 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1493,12 +1493,12 @@
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1609,12 +1609,12 @@
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1667,12 +1667,12 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1725,12 +1725,12 @@
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1899,12 +1899,12 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2073,12 +2073,12 @@
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2131,12 +2131,70 @@
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>20 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>+0.1%</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>+2.7%</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Variación mensual estimada (%)</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Serie desestacionalizada</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>INEGI</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PIBSEC/PIBT: distingue EOPIBT vs PIBT, amplía histórico a 1993 y rediseña fichas.
- Diferencia nombres, siglas y descripciones de EOPIBT (PIB) y PIBT (PIBSEC).
- Extiende el histórico de PIBSEC hasta 1T-1993 con niveles del BIE.
- Calcula variaciones trimestrales/anuales desde niveles históricas y conserva las cifras oficiales desestacionalizadas del boletín PIBT para 2021 en adelante.
- Rediseña la ficha PIBT: 4 small multiples de niveles + 2 gráficas de barras agrupadas de variaciones trimestral/anual.
- Compacta sectores destacados en 3 al alza y 3 a la baja.
- Actualiza tarjetas superiores, lectura ≤4 bullets y responsive.
- Ajusta rangos plausibles en validate.py y mantiene tests verdes.
- Regenera datos, Excel, CSV y summary.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/IOAE/IOAE_datos.xlsx
+++ b/downloads/indicadores/IOAE/IOAE_datos.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -983,18 +983,18 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Nov 24</t>
+          <t>Jul 24</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>45597</v>
+        <v>45474</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>+0.2%</t>
+          <t>-0.1%</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1041,18 +1041,18 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Dic 24</t>
+          <t>Nov 24</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>45627</v>
+        <v>45597</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>+0.4%</t>
+          <t>+0.2%</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1099,18 +1099,18 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Ene 25</t>
+          <t>Dic 24</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>45658</v>
+        <v>45627</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+0.4%</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>+1.8%</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1157,18 +1157,18 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Feb 25</t>
+          <t>Ene 25</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>45689</v>
+        <v>45658</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>+0.2%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>+1.8%</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1215,18 +1215,18 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Mar 25</t>
+          <t>Feb 25</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>45717</v>
+        <v>45689</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>+0.2%</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>-0.2%</t>
+          <t>-0.7%</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1273,11 +1273,11 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Abr 25</t>
+          <t>Mar 25</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45748</v>
+        <v>45717</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>0</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>-0.2%</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1331,18 +1331,18 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>May 25</t>
+          <t>Abr 25</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>45778</v>
+        <v>45748</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>+0.7%</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1389,18 +1389,18 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Jun 25</t>
+          <t>May 25</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45809</v>
+        <v>45778</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>+0.2%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>+1.3%</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1447,18 +1447,18 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Jul 25</t>
+          <t>Jun 25</t>
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>45839</v>
+        <v>45809</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>-0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>-0.1%</t>
+          <t>+0.2%</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1505,28 +1505,28 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Ago 25</t>
+          <t>Jul 25</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>0.1</v>
+        <v>-0.1</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
+          <t>-0.1%</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t>+0.1%</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>+0.2%</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1563,11 +1563,11 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Sep 25</t>
+          <t>Ago 25</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>45901</v>
+        <v>45870</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>0.1</v>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>-0.6%</t>
+          <t>+0.2%</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1621,18 +1621,18 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Oct 25</t>
+          <t>Sep 25</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>45931</v>
+        <v>45901</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-0.6%</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1679,18 +1679,18 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Nov 25</t>
+          <t>Oct 25</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>45962</v>
+        <v>45931</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>-0.2%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1737,18 +1737,18 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Dic 25</t>
+          <t>Nov 25</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>45992</v>
+        <v>45962</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>0.2</v>
+        <v>-0.2</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>+0.2%</t>
+          <t>-0.2%</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>+2.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1795,18 +1795,18 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Ene 26</t>
+          <t>Dic 25</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>46023</v>
+        <v>45992</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>+0.3%</t>
+          <t>+0.2%</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -1853,18 +1853,18 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Feb 26</t>
+          <t>Ene 26</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>46054</v>
+        <v>46023</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+0.3%</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>+2.3%</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1911,18 +1911,18 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Mar 26</t>
+          <t>Feb 26</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>46082</v>
+        <v>46054</v>
       </c>
       <c r="C29" s="9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1969,18 +1969,18 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Abr 26</t>
+          <t>Mar 26</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>46113</v>
+        <v>46082</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>+0.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>+0.3%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2027,18 +2027,18 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Abr 26</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="C31" s="9" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>+0.3%</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>+0.3%</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -2085,18 +2085,18 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Jun 26</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>+0.2%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>+1.7%</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2143,56 +2143,114 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>+1.7%</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Variación mensual estimada (%)</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Serie desestacionalizada</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>INEGI</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>20 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B33" s="8" t="n">
+      <c r="B34" s="5" t="n">
         <v>46204</v>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C34" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>+0.1%</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>+2.7%</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>Variación mensual estimada (%)</t>
-        </is>
-      </c>
-      <c r="H33" s="7" t="inlineStr">
-        <is>
-          <t>Serie desestacionalizada</t>
-        </is>
-      </c>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>Definitivo</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>INEGI</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
-        </is>
-      </c>
-      <c r="L33" s="7" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Variación mensual estimada (%)</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Serie desestacionalizada</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>INEGI</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ioae/ioae2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>20 de agosto de 2026</t>
         </is>

</xml_diff>